<commit_message>
Correction of datetime format
</commit_message>
<xml_diff>
--- a/output/tables/spo2_12h_by_treatment_obs.xlsx
+++ b/output/tables/spo2_12h_by_treatment_obs.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t xml:space="preserve">Time Since Randomisation (hours)
 </t>
@@ -44,103 +44,106 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">1,180</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92.79 (3.32)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">94.86 (3.30)</t>
+    <t xml:space="preserve">93.73 (3.32)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.71 (3.65)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.85, -0.65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;0.001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92.17 (3.06)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.98 (2.89)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.15, -2.60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92.11 (2.95)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.91 (2.92)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.30, -2.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">91.93 (2.54)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.73 (2.69)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.28, -2.79</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92.29 (2.41)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.28 (2.74)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.55, -2.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92.05 (2.90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.20 (3.01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-3.00, -2.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92.16 (2.88)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.24 (2.64)</t>
   </si>
   <si>
     <t xml:space="preserve">-2.75, -2.00</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;0.001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92.19 (2.55)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">94.69 (2.87)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3.00, -2.20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92.00 (2.98)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">94.89 (2.76)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3.45, -2.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92.15 (2.34)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">94.54 (2.72)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-3.00, -2.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92.04 (2.87)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">94.08 (2.74)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.85, -2.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92.05 (2.88)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">94.09 (3.02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92.31 (2.87)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">93.77 (2.62)</t>
+    <t xml:space="preserve">92.08 (2.83)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93.72 (2.98)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.00, -1.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92.75 (3.05)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.03 (2.81)</t>
   </si>
   <si>
     <t xml:space="preserve">-2.00, -1.00</t>
   </si>
   <si>
-    <t xml:space="preserve">92.48 (2.91)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">93.93 (2.81)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92.61 (3.14)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">94.40 (2.90)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.65, -1.60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">92.38 (2.73)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">93.52 (3.19)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.00, -0.60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">93.52 (2.77)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">94.94 (2.70)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2.10, -1.00</t>
+    <t xml:space="preserve">92.38 (3.03)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.06 (2.86)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.20, -1.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">92.90 (2.79)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">94.07 (3.12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-2.00, -0.90</t>
   </si>
   <si>
     <t xml:space="preserve">Mean (SD)</t>
@@ -622,23 +625,23 @@
       <c r="A2" s="2" t="n">
         <v>-12</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="7" t="n">
+        <v>483</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="E2" s="7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="7" t="n">
-        <v>-2.05</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>10</v>
-      </c>
       <c r="G2" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" ht="NA" customHeight="1">
@@ -646,22 +649,22 @@
         <v>0</v>
       </c>
       <c r="B3" s="8" t="n">
-        <v>828</v>
+        <v>773</v>
       </c>
       <c r="C3" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" s="8" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="8" t="n">
-        <v>-2.85</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>14</v>
-      </c>
       <c r="G3" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" ht="NA" customHeight="1">
@@ -669,22 +672,22 @@
         <v>12</v>
       </c>
       <c r="B4" s="8" t="n">
-        <v>703</v>
+        <v>767</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>15</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>16</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>-3</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" ht="NA" customHeight="1">
@@ -692,22 +695,22 @@
         <v>24</v>
       </c>
       <c r="B5" s="8" t="n">
-        <v>828</v>
+        <v>765</v>
       </c>
       <c r="C5" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E5" s="8" t="n">
+        <v>-3</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="8" t="n">
-        <v>-2.6</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>20</v>
-      </c>
       <c r="G5" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" ht="NA" customHeight="1">
@@ -715,22 +718,22 @@
         <v>36</v>
       </c>
       <c r="B6" s="8" t="n">
-        <v>689</v>
+        <v>783</v>
       </c>
       <c r="C6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="E6" s="8" t="n">
+        <v>-2</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="8" t="n">
-        <v>-2.1</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>23</v>
-      </c>
       <c r="G6" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" ht="NA" customHeight="1">
@@ -738,22 +741,22 @@
         <v>48</v>
       </c>
       <c r="B7" s="8" t="n">
-        <v>800</v>
+        <v>738</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="E7" s="8" t="n">
+        <v>-2.25</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="8" t="n">
-        <v>-2</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>10</v>
-      </c>
       <c r="G7" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="NA" customHeight="1">
@@ -761,7 +764,7 @@
         <v>60</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>647</v>
+        <v>750</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>26</v>
@@ -770,13 +773,13 @@
         <v>27</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>-1.4</v>
+        <v>-2</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>28</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" ht="NA" customHeight="1">
@@ -784,7 +787,7 @@
         <v>72</v>
       </c>
       <c r="B9" s="8" t="n">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>29</v>
@@ -793,13 +796,13 @@
         <v>30</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>-1.6</v>
+        <v>-1.95</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10" ht="NA" customHeight="1">
@@ -807,22 +810,22 @@
         <v>84</v>
       </c>
       <c r="B10" s="8" t="n">
-        <v>594</v>
+        <v>647</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>-2</v>
+        <v>-1.3</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" ht="NA" customHeight="1">
@@ -830,22 +833,22 @@
         <v>96</v>
       </c>
       <c r="B11" s="8" t="n">
-        <v>366</v>
+        <v>590</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" ht="NA" customHeight="1">
@@ -853,91 +856,91 @@
         <v>108</v>
       </c>
       <c r="B12" s="9" t="n">
-        <v>205</v>
+        <v>541</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>-1.85</v>
+        <v>-1.05</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" ht="NA" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" ht="NA" customHeight="1">
       <c r="A14" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" ht="NA" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>